<commit_message>
add files referenced by figures/
</commit_message>
<xml_diff>
--- a/data/20260413_anthracnoseResistanceCandidates.xlsx
+++ b/data/20260413_anthracnoseResistanceCandidates.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jensinadavis/Documents/fieldLeafImaging/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11631FFB-98EC-2E4A-9F3B-D6967E16F0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D96EC00D-566F-9A49-92F5-4855EE88DE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{7DF28695-A593-A44A-AF17-F68326F142C9}"/>
+    <workbookView xWindow="68640" yWindow="480" windowWidth="38400" windowHeight="21120" activeTab="2" xr2:uid="{7DF28695-A593-A44A-AF17-F68326F142C9}"/>
   </bookViews>
   <sheets>
     <sheet name="20260224_genes_markers_Cs_JD" sheetId="1" r:id="rId1"/>
     <sheet name="candidates" sheetId="2" r:id="rId2"/>
+    <sheet name="validated_all_diseases" sheetId="3" r:id="rId3"/>
+    <sheet name="candidates_all_diseases" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20260224_genes_markers_Cs_JD'!$A$1:$I$32</definedName>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="427">
   <si>
     <t>Gene ID</t>
   </si>
@@ -861,13 +863,462 @@
   </si>
   <si>
     <t>Sobic.009G221266</t>
+  </si>
+  <si>
+    <t>Disease</t>
+  </si>
+  <si>
+    <t>Turcicum leaf blight</t>
+  </si>
+  <si>
+    <t>Expression induction and VIGS of the cluster increased susceptibility</t>
+  </si>
+  <si>
+    <t>Martin et al. (2011)</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/1471-2229-11-151</t>
+  </si>
+  <si>
+    <t>Sobic.005G095700</t>
+  </si>
+  <si>
+    <t>Sobic.005G096300</t>
+  </si>
+  <si>
+    <t>Sobic.005G092600</t>
+  </si>
+  <si>
+    <t>Sobic.005G095000</t>
+  </si>
+  <si>
+    <t>Sobic.005G095600</t>
+  </si>
+  <si>
+    <t>Sobic.002G058400</t>
+  </si>
+  <si>
+    <t>RPM1 like NLR near a significant GWAS peak, no functional validation</t>
+  </si>
+  <si>
+    <t>Birhanu et al. (2024)</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1186/s12864-024-10545-2</t>
+  </si>
+  <si>
+    <t>Sobic.004G326400</t>
+  </si>
+  <si>
+    <t>Xa21 binding receptor like kinase candidate sits in the lead SNP interval, still association based</t>
+  </si>
+  <si>
+    <t>Sobic.008G156600</t>
+  </si>
+  <si>
+    <t>LRR family protein within local LD, not functionally tested</t>
+  </si>
+  <si>
+    <t>Sobic.008G157400</t>
+  </si>
+  <si>
+    <t>NB ARC candidate within local LD, not functionally tested</t>
+  </si>
+  <si>
+    <t>Sobic.002G022600</t>
+  </si>
+  <si>
+    <t>Wall associated kinase candidate in the LD block, no functional test</t>
+  </si>
+  <si>
+    <t>Sobic.005G160400</t>
+  </si>
+  <si>
+    <t>Sobic.005G164200</t>
+  </si>
+  <si>
+    <t>Sobic.005G164300</t>
+  </si>
+  <si>
+    <t>Sobic.005G167600</t>
+  </si>
+  <si>
+    <t>Sobic.005G169200</t>
+  </si>
+  <si>
+    <t>Sobic.005G169300</t>
+  </si>
+  <si>
+    <t>Sobic.005G169400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sobic.005G177400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sobic.005G177500</t>
+  </si>
+  <si>
+    <t>Sobic.005G177600</t>
+  </si>
+  <si>
+    <t>Sobic.005G181700</t>
+  </si>
+  <si>
+    <t>Sobic.005G182800</t>
+  </si>
+  <si>
+    <t>Sobic.005G183700</t>
+  </si>
+  <si>
+    <t>Sobic.005G183900</t>
+  </si>
+  <si>
+    <t>Sobic.005G186100</t>
+  </si>
+  <si>
+    <t>Sobic.005G192600</t>
+  </si>
+  <si>
+    <t>Sobic.005G193600</t>
+  </si>
+  <si>
+    <t>Sobic.005G195000</t>
+  </si>
+  <si>
+    <t>Sobic.005G209000</t>
+  </si>
+  <si>
+    <t>Sobic.005G209100</t>
+  </si>
+  <si>
+    <t>Sobic.005G212700</t>
+  </si>
+  <si>
+    <t>Sobic.005G213500</t>
+  </si>
+  <si>
+    <t>Sobic.005G219300</t>
+  </si>
+  <si>
+    <t>Sobic.005G220300</t>
+  </si>
+  <si>
+    <t>Sobic.005G223700</t>
+  </si>
+  <si>
+    <t>Sobic.005G224000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sobic.005G224200</t>
+  </si>
+  <si>
+    <t>Sobic.005G224900</t>
+  </si>
+  <si>
+    <t>Sobic.005G226100</t>
+  </si>
+  <si>
+    <t>Sobic.005G226200</t>
+  </si>
+  <si>
+    <t>Sobic.005G226500</t>
+  </si>
+  <si>
+    <t>Sobic.005G229400</t>
+  </si>
+  <si>
+    <t>Sobic.005G229600</t>
+  </si>
+  <si>
+    <t>Under major anthracnose resistance QTL with LOD score &gt; 3.9 threshold and have disease, defense, or wound response associated GO terms</t>
+  </si>
+  <si>
+    <t>Burrell et al. (2015)</t>
+  </si>
+  <si>
+    <t>https://acsess.onlinelibrary.wiley.com/doi/abs/10.2135/cropsci2014.06.0430?casa_token=11q7hH9NijcAAAAA%3Arr3HAbnwi5FUd21J-Vt2-xHtHY9GubRvApKsNEI7QIw5lw3f1aeF5yvI-W_oTrMjFbrT03GJ6HhpHCQ</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1007/s00122-013-2081-1/tables/1</t>
+  </si>
+  <si>
+    <t>Upadhyaya et al. (2013)</t>
+  </si>
+  <si>
+    <t>Under GWAS peak with disease resistance annotations or homology</t>
+  </si>
+  <si>
+    <t>Sobic.006G158600</t>
+  </si>
+  <si>
+    <t>Sobic.006G158800</t>
+  </si>
+  <si>
+    <t>Sobic.006G159000</t>
+  </si>
+  <si>
+    <t>Sobic.006G158900</t>
+  </si>
+  <si>
+    <t>Sobic.001G242600</t>
+  </si>
+  <si>
+    <t>Sobic.001G528200</t>
+  </si>
+  <si>
+    <t>Sobic.008G042900</t>
+  </si>
+  <si>
+    <t>Sobic.008G043000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sobic.008G043100</t>
+  </si>
+  <si>
+    <t>Sobic.001G122000</t>
+  </si>
+  <si>
+    <t>Sobic.001G298300</t>
+  </si>
+  <si>
+    <t>https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0216671</t>
+  </si>
+  <si>
+    <t>Nearest gene to MLM peak SNP</t>
+  </si>
+  <si>
+    <t>Ahn et al. (2019)</t>
+  </si>
+  <si>
+    <t>Sobic.008G020700</t>
+  </si>
+  <si>
+    <t>Sobic.002G330900</t>
+  </si>
+  <si>
+    <t>Sobic.004G273600</t>
+  </si>
+  <si>
+    <t>Sobic.007G105400</t>
+  </si>
+  <si>
+    <t>Sobic.003G281500</t>
+  </si>
+  <si>
+    <t>Sobic.005G024400</t>
+  </si>
+  <si>
+    <t>Sobic.006G040101</t>
+  </si>
+  <si>
+    <t>Sobic.001G097400</t>
+  </si>
+  <si>
+    <t>Sobic.003G325100</t>
+  </si>
+  <si>
+    <t>Sobic.009G082200</t>
+  </si>
+  <si>
+    <t>disease</t>
+  </si>
+  <si>
+    <t>Downy mildew</t>
+  </si>
+  <si>
+    <t>Sobic.001G339100</t>
+  </si>
+  <si>
+    <t>Sobic.003G185000</t>
+  </si>
+  <si>
+    <t>Sobic.003G018300</t>
+  </si>
+  <si>
+    <t>Sobic.002G249000</t>
+  </si>
+  <si>
+    <t>Sobic.010G126500</t>
+  </si>
+  <si>
+    <t>Sobic.003G018600</t>
+  </si>
+  <si>
+    <t>Sobic.001G111300</t>
+  </si>
+  <si>
+    <t>Sobic.004G289700</t>
+  </si>
+  <si>
+    <t>Sobic.002G224300</t>
+  </si>
+  <si>
+    <t>Sobic.001G105900</t>
+  </si>
+  <si>
+    <t>Head smut</t>
+  </si>
+  <si>
+    <t>Sobic.001G459500</t>
+  </si>
+  <si>
+    <t>Sobic.003G207500</t>
+  </si>
+  <si>
+    <t>Sobic.005G049600</t>
+  </si>
+  <si>
+    <t>Sobic.010G143900</t>
+  </si>
+  <si>
+    <t>Sobic.002G142900</t>
+  </si>
+  <si>
+    <t>Sobic.005G076301</t>
+  </si>
+  <si>
+    <t>Sobic.002G019000</t>
+  </si>
+  <si>
+    <t>Sobic.005G120201</t>
+  </si>
+  <si>
+    <t>Sobic.001G459600</t>
+  </si>
+  <si>
+    <t>Sobic.006G160500</t>
+  </si>
+  <si>
+    <t>Sobic.002G007800</t>
+  </si>
+  <si>
+    <t>Leaf blight</t>
+  </si>
+  <si>
+    <t>Sobic.009G099450</t>
+  </si>
+  <si>
+    <t>Sobic.003G351501</t>
+  </si>
+  <si>
+    <t>Sobic.008G070700</t>
+  </si>
+  <si>
+    <t>Sobic.009G057200</t>
+  </si>
+  <si>
+    <t>Sobic.002G147900</t>
+  </si>
+  <si>
+    <t>Sorghum smut</t>
+  </si>
+  <si>
+    <t>Ahn et al. (2022)</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2223-7747/11/21/2999</t>
+  </si>
+  <si>
+    <t>Sobic.004G202700</t>
+  </si>
+  <si>
+    <t>Sobic.002G174700</t>
+  </si>
+  <si>
+    <t>Sobic.004G273200</t>
+  </si>
+  <si>
+    <t>Sobic.004G319800</t>
+  </si>
+  <si>
+    <t>Sobic.003G427400</t>
+  </si>
+  <si>
+    <t>Sobic.001G430000</t>
+  </si>
+  <si>
+    <t>Sobic.002G174300</t>
+  </si>
+  <si>
+    <t>Stalk rot diseases</t>
+  </si>
+  <si>
+    <t>https://academic.oup.com/g3journal/article/5/6/1165/6025270?guestAccessKey=</t>
+  </si>
+  <si>
+    <t>Adeyanju et al. (2015)</t>
+  </si>
+  <si>
+    <t>Sobic.009G241000</t>
+  </si>
+  <si>
+    <t>Sobic.009G229900</t>
+  </si>
+  <si>
+    <t>Sobic.009G233000</t>
+  </si>
+  <si>
+    <t>Sobic.007G140900</t>
+  </si>
+  <si>
+    <t>Sobic.002G261500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Sobic.002G209600</t>
+  </si>
+  <si>
+    <t>Sobic.007G163500</t>
+  </si>
+  <si>
+    <t>Sobic.009G232300</t>
+  </si>
+  <si>
+    <t>Sobic.002G145400</t>
+  </si>
+  <si>
+    <t>Sobic.003G099100</t>
+  </si>
+  <si>
+    <t>Sobic.009G224200</t>
+  </si>
+  <si>
+    <t>Sobic.004G332000</t>
+  </si>
+  <si>
+    <t>Sobic.008G154100</t>
+  </si>
+  <si>
+    <t>Sobic.008G098200</t>
+  </si>
+  <si>
+    <t>Xanthomonas &amp; Psuedomonas</t>
+  </si>
+  <si>
+    <t>VIGs targeting the gene increases susceptibility.</t>
+  </si>
+  <si>
+    <t>Bredow et al. (2023)</t>
+  </si>
+  <si>
+    <t>https://bsppjournals.onlinelibrary.wiley.com/doi/10.1111/mpp.13270</t>
+  </si>
+  <si>
+    <t>Sobic.001G033400</t>
+  </si>
+  <si>
+    <t>Sobic.001G421300</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1014,6 +1465,44 @@
       <color rgb="FF222222"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color rgb="FF5A5A5A"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF222222"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1B1B1B"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1313,7 +1802,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1356,13 +1845,23 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1396,6 +1895,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -1420,9 +1920,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1460,7 +1960,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1566,7 +2066,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1708,7 +2208,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2482,11 +2982,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F0639B-AA9C-CB4E-A0BF-98F3E878491E}">
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D155"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" customWidth="1"/>
     <col min="2" max="2" width="30.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -3737,8 +4238,1894 @@
         <v>269</v>
       </c>
     </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C94" t="s">
+        <v>291</v>
+      </c>
+      <c r="D94" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C95" t="s">
+        <v>291</v>
+      </c>
+      <c r="D95" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C96" t="s">
+        <v>291</v>
+      </c>
+      <c r="D96" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C97" t="s">
+        <v>291</v>
+      </c>
+      <c r="D97" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="C98" t="s">
+        <v>291</v>
+      </c>
+      <c r="D98" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>301</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C99" t="s">
+        <v>335</v>
+      </c>
+      <c r="D99" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A100" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C100" t="s">
+        <v>335</v>
+      </c>
+      <c r="D100" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A101" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C101" t="s">
+        <v>335</v>
+      </c>
+      <c r="D101" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A102" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C102" t="s">
+        <v>335</v>
+      </c>
+      <c r="D102" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A103" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C103" t="s">
+        <v>335</v>
+      </c>
+      <c r="D103" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>306</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C104" t="s">
+        <v>335</v>
+      </c>
+      <c r="D104" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A105" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C105" t="s">
+        <v>335</v>
+      </c>
+      <c r="D105" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C106" t="s">
+        <v>335</v>
+      </c>
+      <c r="D106" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A107" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C107" t="s">
+        <v>335</v>
+      </c>
+      <c r="D107" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A108" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C108" t="s">
+        <v>335</v>
+      </c>
+      <c r="D108" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A109" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C109" t="s">
+        <v>335</v>
+      </c>
+      <c r="D109" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A110" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C110" t="s">
+        <v>335</v>
+      </c>
+      <c r="D110" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A111" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C111" t="s">
+        <v>335</v>
+      </c>
+      <c r="D111" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A112" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C112" t="s">
+        <v>335</v>
+      </c>
+      <c r="D112" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A113" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C113" t="s">
+        <v>335</v>
+      </c>
+      <c r="D113" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A114" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C114" t="s">
+        <v>335</v>
+      </c>
+      <c r="D114" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A115" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C115" t="s">
+        <v>335</v>
+      </c>
+      <c r="D115" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A116" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C116" t="s">
+        <v>335</v>
+      </c>
+      <c r="D116" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A117" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C117" t="s">
+        <v>335</v>
+      </c>
+      <c r="D117" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A118" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C118" t="s">
+        <v>335</v>
+      </c>
+      <c r="D118" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A119" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C119" t="s">
+        <v>335</v>
+      </c>
+      <c r="D119" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A120" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C120" t="s">
+        <v>335</v>
+      </c>
+      <c r="D120" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A121" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C121" t="s">
+        <v>335</v>
+      </c>
+      <c r="D121" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A122" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C122" t="s">
+        <v>335</v>
+      </c>
+      <c r="D122" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A123" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C123" t="s">
+        <v>335</v>
+      </c>
+      <c r="D123" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A124" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C124" t="s">
+        <v>335</v>
+      </c>
+      <c r="D124" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A125" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C125" t="s">
+        <v>335</v>
+      </c>
+      <c r="D125" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A126" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C126" t="s">
+        <v>335</v>
+      </c>
+      <c r="D126" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A127" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C127" t="s">
+        <v>335</v>
+      </c>
+      <c r="D127" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A128" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C128" t="s">
+        <v>335</v>
+      </c>
+      <c r="D128" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A129" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C129" t="s">
+        <v>335</v>
+      </c>
+      <c r="D129" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A130" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C130" t="s">
+        <v>335</v>
+      </c>
+      <c r="D130" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A131" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C131" t="s">
+        <v>335</v>
+      </c>
+      <c r="D131" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A132" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C132" t="s">
+        <v>335</v>
+      </c>
+      <c r="D132" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A133" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C133" t="s">
+        <v>335</v>
+      </c>
+      <c r="D133" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A134" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C134" t="s">
+        <v>335</v>
+      </c>
+      <c r="D134" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A135" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D135" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A136" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D136" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A137" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D137" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A138" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D138" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A139" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D139" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A140" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D140" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A141" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D141" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A142" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D142" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A143" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D143" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A144" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D144" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" ht="19" x14ac:dyDescent="0.2">
+      <c r="A145" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D145" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A146" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="B146" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D146" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A147" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C147" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D147" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A148" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C148" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D148" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A149" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="B149" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C149" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D149" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A150" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="B150" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C150" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D150" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A151" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C151" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D151" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A152" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B152" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C152" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D152" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A153" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B153" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C153" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D153" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A154" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B154" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D154" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A155" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D155" t="s">
+        <v>351</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E26AF127-4B8F-9245-BFFE-32ED406A07E3}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B4" t="s">
+        <v>286</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D4" t="s">
+        <v>282</v>
+      </c>
+      <c r="E4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>280</v>
+      </c>
+      <c r="B5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E5" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" t="s">
+        <v>282</v>
+      </c>
+      <c r="E6" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>421</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="D7" t="s">
+        <v>423</v>
+      </c>
+      <c r="E7" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>421</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="D8" t="s">
+        <v>423</v>
+      </c>
+      <c r="E8" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>421</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="D9" t="s">
+        <v>423</v>
+      </c>
+      <c r="E9" t="s">
+        <v>424</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D27D09B6-FAAF-0D46-BEED-DFC4393D5EA0}">
+  <dimension ref="A1:E49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D3" t="s">
+        <v>351</v>
+      </c>
+      <c r="E3" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D5" t="s">
+        <v>351</v>
+      </c>
+      <c r="E5" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
+        <v>370</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D6" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E7" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
+        <v>372</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D8" t="s">
+        <v>351</v>
+      </c>
+      <c r="E8" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D9" t="s">
+        <v>351</v>
+      </c>
+      <c r="E9" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D10" t="s">
+        <v>351</v>
+      </c>
+      <c r="E10" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D11" t="s">
+        <v>351</v>
+      </c>
+      <c r="E11" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D12" t="s">
+        <v>351</v>
+      </c>
+      <c r="E12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D13" t="s">
+        <v>351</v>
+      </c>
+      <c r="E13" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D14" t="s">
+        <v>351</v>
+      </c>
+      <c r="E14" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D15" t="s">
+        <v>351</v>
+      </c>
+      <c r="E15" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D16" t="s">
+        <v>351</v>
+      </c>
+      <c r="E16" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D17" t="s">
+        <v>351</v>
+      </c>
+      <c r="E17" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D18" t="s">
+        <v>351</v>
+      </c>
+      <c r="E18" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D19" t="s">
+        <v>351</v>
+      </c>
+      <c r="E19" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D20" t="s">
+        <v>351</v>
+      </c>
+      <c r="E20" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D21" t="s">
+        <v>351</v>
+      </c>
+      <c r="E21" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D22" t="s">
+        <v>351</v>
+      </c>
+      <c r="E22" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D23" t="s">
+        <v>351</v>
+      </c>
+      <c r="E23" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D24" t="s">
+        <v>351</v>
+      </c>
+      <c r="E24" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D25" t="s">
+        <v>351</v>
+      </c>
+      <c r="E25" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D26" t="s">
+        <v>351</v>
+      </c>
+      <c r="E26" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D27" t="s">
+        <v>351</v>
+      </c>
+      <c r="E27" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D28" t="s">
+        <v>396</v>
+      </c>
+      <c r="E28" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D29" t="s">
+        <v>396</v>
+      </c>
+      <c r="E29" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D30" t="s">
+        <v>396</v>
+      </c>
+      <c r="E30" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D31" t="s">
+        <v>396</v>
+      </c>
+      <c r="E31" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D32" t="s">
+        <v>396</v>
+      </c>
+      <c r="E32" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D33" t="s">
+        <v>396</v>
+      </c>
+      <c r="E33" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="D34" t="s">
+        <v>396</v>
+      </c>
+      <c r="E34" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E35" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E36" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E37" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E38" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E39" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E40" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E41" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E42" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E43" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E44" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E45" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E46" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E47" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="19" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E48" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="E49" t="s">
+        <v>404</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D35" r:id="rId1" xr:uid="{B5C65C54-E20A-BA4D-9702-A2360CC755DF}"/>
+    <hyperlink ref="D36:D49" r:id="rId2" display="https://academic.oup.com/g3journal/article/5/6/1165/6025270?guestAccessKey=" xr:uid="{0D0A988D-D533-1C4B-9D4A-D44714DD39B1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>